<commit_message>
doc and excel updated
</commit_message>
<xml_diff>
--- a/Bank_Results.xlsx
+++ b/Bank_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\BankParser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0CBABAD-F118-4F56-9D2C-CAA47C3E23BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{803116C6-BEB4-48D2-8012-51D3ABF14A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CE7BBC11-F063-4F4E-8401-6E769C3C185D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="43">
   <si>
     <t xml:space="preserve">Bank Name </t>
   </si>
@@ -80,9 +80,6 @@
     <t xml:space="preserve">Account number not getting split by Suffix </t>
   </si>
   <si>
-    <t>Multi Account /Row Parser</t>
-  </si>
-  <si>
     <t>Mismatch in debit and interest amount ot be seperated</t>
   </si>
   <si>
@@ -152,10 +149,22 @@
     <t>Ascend Bank</t>
   </si>
   <si>
-    <t>Multi Account /Debit Credit Row Parser</t>
-  </si>
-  <si>
     <t xml:space="preserve">Account number not getting split by ID0000 </t>
+  </si>
+  <si>
+    <t>SingleMulti Account -Row Parser</t>
+  </si>
+  <si>
+    <t>Multi Account -Row Parser</t>
+  </si>
+  <si>
+    <t>Single Account -Row Parser</t>
+  </si>
+  <si>
+    <t>Single Account-Section Parser</t>
+  </si>
+  <si>
+    <t>Multi Account -Debit Credit Row Parser</t>
   </si>
 </sst>
 </file>
@@ -324,20 +333,20 @@
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:from>
         <xdr:to>
-          <xdr:col>12</xdr:col>
-          <xdr:colOff>228600</xdr:colOff>
-          <xdr:row>30</xdr:row>
-          <xdr:rowOff>38100</xdr:rowOff>
+          <xdr:col>5</xdr:col>
+          <xdr:colOff>914400</xdr:colOff>
+          <xdr:row>2</xdr:row>
+          <xdr:rowOff>320040</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="1026" name="Object 2" hidden="1">
+            <xdr:cNvPr id="1027" name="Object 3" hidden="1">
               <a:extLst>
                 <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
-                  <a14:compatExt spid="_x0000_s1026"/>
+                  <a14:compatExt spid="_x0000_s1027"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{423ED2EA-47C6-5E28-2733-F21795638070}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96E64A97-65DC-3A27-121E-B3C15CDF5D0A}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -741,7 +750,7 @@
         <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D2" s="5" t="s">
         <v>12</v>
@@ -757,7 +766,7 @@
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>8</v>
@@ -767,29 +776,29 @@
     </row>
     <row r="4" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
     </row>
     <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>13</v>
@@ -799,58 +808,58 @@
     </row>
     <row r="6" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
     </row>
     <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
     </row>
     <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="D8" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
     </row>
     <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
         <v>7</v>
@@ -860,10 +869,10 @@
     </row>
     <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
@@ -873,80 +882,80 @@
     </row>
     <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="C13" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
     </row>
     <row r="14" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="C14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
     </row>
     <row r="15" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>37</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -1004,7 +1013,7 @@
     </mc:AlternateContent>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice Requires="x14">
-        <oleObject progId="Document" shapeId="1026" r:id="rId6">
+        <oleObject progId="Document" dvAspect="DVASPECT_ICON" shapeId="1027" r:id="rId6">
           <objectPr defaultSize="0" r:id="rId7">
             <anchor moveWithCells="1">
               <from>
@@ -1014,17 +1023,17 @@
                 <xdr:rowOff>0</xdr:rowOff>
               </from>
               <to>
-                <xdr:col>12</xdr:col>
-                <xdr:colOff>228600</xdr:colOff>
-                <xdr:row>30</xdr:row>
-                <xdr:rowOff>38100</xdr:rowOff>
+                <xdr:col>5</xdr:col>
+                <xdr:colOff>914400</xdr:colOff>
+                <xdr:row>2</xdr:row>
+                <xdr:rowOff>320040</xdr:rowOff>
               </to>
             </anchor>
           </objectPr>
         </oleObject>
       </mc:Choice>
       <mc:Fallback>
-        <oleObject progId="Document" shapeId="1026" r:id="rId6"/>
+        <oleObject progId="Document" dvAspect="DVASPECT_ICON" shapeId="1027" r:id="rId6"/>
       </mc:Fallback>
     </mc:AlternateContent>
   </oleObjects>

</xml_diff>

<commit_message>
pending bank configuration added
</commit_message>
<xml_diff>
--- a/Bank_Results.xlsx
+++ b/Bank_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\BankParser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{803116C6-BEB4-48D2-8012-51D3ABF14A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4B9D0B2-B52A-49C8-AF83-EF5D7B7C24A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CE7BBC11-F063-4F4E-8401-6E769C3C185D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="45">
   <si>
     <t xml:space="preserve">Bank Name </t>
   </si>
@@ -119,9 +119,6 @@
     <t>Start and End balance to be mapped correctly</t>
   </si>
   <si>
-    <t xml:space="preserve">Account number not getting split by Acc# </t>
-  </si>
-  <si>
     <t>DCU Bank</t>
   </si>
   <si>
@@ -149,9 +146,6 @@
     <t>Ascend Bank</t>
   </si>
   <si>
-    <t xml:space="preserve">Account number not getting split by ID0000 </t>
-  </si>
-  <si>
     <t>SingleMulti Account -Row Parser</t>
   </si>
   <si>
@@ -165,6 +159,18 @@
   </si>
   <si>
     <t>Multi Account -Debit Credit Row Parser</t>
+  </si>
+  <si>
+    <t>American Heritage Bank</t>
+  </si>
+  <si>
+    <t>Multi Account - Row Parser</t>
+  </si>
+  <si>
+    <t>Working fine with multi account</t>
+  </si>
+  <si>
+    <t>Account split is happening, but unknown split section also getting created which need to be corrected</t>
   </si>
 </sst>
 </file>
@@ -776,10 +782,10 @@
     </row>
     <row r="4" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
         <v>18</v>
@@ -792,10 +798,10 @@
     </row>
     <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
@@ -811,7 +817,7 @@
         <v>17</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C6" t="s">
         <v>19</v>
@@ -827,7 +833,7 @@
         <v>16</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
         <v>22</v>
@@ -843,7 +849,7 @@
         <v>21</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
         <v>22</v>
@@ -856,10 +862,10 @@
     </row>
     <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C9" t="s">
         <v>7</v>
@@ -869,10 +875,10 @@
     </row>
     <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
         <v>7</v>
@@ -882,10 +888,10 @@
     </row>
     <row r="11" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
         <v>22</v>
@@ -898,10 +904,10 @@
     </row>
     <row r="12" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C12" t="s">
         <v>22</v>
@@ -914,10 +920,10 @@
     </row>
     <row r="13" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C13" t="s">
         <v>22</v>
@@ -928,38 +934,46 @@
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
     </row>
-    <row r="14" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
         <v>22</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
     </row>
-    <row r="15" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
         <v>22</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C16" s="3"/>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C16" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="17" spans="3:3" x14ac:dyDescent="0.3">
       <c r="C17" s="3"/>

</xml_diff>

<commit_message>
deduplication code added with some pending changes
</commit_message>
<xml_diff>
--- a/Bank_Results.xlsx
+++ b/Bank_Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\BankParser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4B9D0B2-B52A-49C8-AF83-EF5D7B7C24A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A44CDD00-F766-4689-88A0-2F375F1C9FF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CE7BBC11-F063-4F4E-8401-6E769C3C185D}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="50">
   <si>
     <t xml:space="preserve">Bank Name </t>
   </si>
@@ -171,6 +172,21 @@
   </si>
   <si>
     <t>Account split is happening, but unknown split section also getting created which need to be corrected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Associated Bank </t>
+  </si>
+  <si>
+    <t>Single account - Section Parser</t>
+  </si>
+  <si>
+    <t>Extracted text is getting repetition, could be issue with digitally uploaded document</t>
+  </si>
+  <si>
+    <t>Wafd Bank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No identifiers exists </t>
   </si>
 </sst>
 </file>
@@ -241,7 +257,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -284,7 +300,7 @@
                   <a14:compatExt spid="_x0000_s1025"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{572A6814-43F1-CEF5-5393-F34F97E11880}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000001040000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -305,23 +321,10 @@
               <a:solidFill>
                 <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
               </a:solidFill>
-              <a:prstDash val="solid"/>
               <a:miter lim="800000"/>
               <a:headEnd/>
-              <a:tailEnd type="none" w="med" len="med"/>
+              <a:tailEnd/>
             </a:ln>
-            <a:effectLst/>
-            <a:extLst>
-              <a:ext uri="{AF507438-7753-43E0-B8FC-AC1667EBCBE1}">
-                <a14:hiddenEffects>
-                  <a:effectLst>
-                    <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="808080"/>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </a14:hiddenEffects>
-              </a:ext>
-            </a:extLst>
           </xdr:spPr>
         </xdr:sp>
         <xdr:clientData/>
@@ -352,7 +355,7 @@
                   <a14:compatExt spid="_x0000_s1027"/>
                 </a:ext>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96E64A97-65DC-3A27-121E-B3C15CDF5D0A}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003040000}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -373,23 +376,10 @@
               <a:solidFill>
                 <a:srgbClr val="000000" mc:Ignorable="a14" a14:legacySpreadsheetColorIndex="64"/>
               </a:solidFill>
-              <a:prstDash val="solid"/>
               <a:miter lim="800000"/>
               <a:headEnd/>
-              <a:tailEnd type="none" w="med" len="med"/>
+              <a:tailEnd/>
             </a:ln>
-            <a:effectLst/>
-            <a:extLst>
-              <a:ext uri="{AF507438-7753-43E0-B8FC-AC1667EBCBE1}">
-                <a14:hiddenEffects>
-                  <a:effectLst>
-                    <a:outerShdw dist="35921" dir="2700000" algn="ctr" rotWithShape="0">
-                      <a:srgbClr val="808080"/>
-                    </a:outerShdw>
-                  </a:effectLst>
-                </a14:hiddenEffects>
-              </a:ext>
-            </a:extLst>
           </xdr:spPr>
         </xdr:sp>
         <xdr:clientData/>
@@ -975,19 +965,38 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C17" s="3"/>
-    </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C18" s="3"/>
-    </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C19" s="3"/>
     </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C20" s="3"/>
     </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C21" s="4"/>
     </row>
   </sheetData>

</xml_diff>